<commit_message>
Append PDF text to template headers instead of overwriting
- Add `handling` field to ExtractedData for section 7.1
- Map handling_1 to A54 and storage_1 to A55
- Implement append mode in write_value with rich text support
- Preserve bold headers and append PDF content in normal Arial font
- Strip "z pkt. X.Y KCH" placeholders from template headers
- Update template with bold headers in A41-A44, A48-A50, A54-A55

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wzor.xlsx
+++ b/wzor.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t>INSTRUKCJA BHP
 PRZY STOSOWANIU MIESZANIN 
@@ -87,6 +87,176 @@
     <t>Pierwsza pomoc</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Uwagi ogólne:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>w</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>razie wypadku z użyciem środka każdorazowo sprawdzić szczegółowe metody udzielania pierwszej pomocy w kartach charakterystyki poszczególnych środków:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">z pkt. 4.2 KCH. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Drogi oddechowe: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">z pkt. 4.2 KCH. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Kontakt ze skórą:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">z pkt. 4.2 KCH. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Kontakt z oczami:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">z pkt. 4.2 KCH. </t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Drogi pokarmowe: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve">z pkt. 4.2 KCH. </t>
+    </r>
+  </si>
+  <si>
     <t>POGOTOWIE RATUNKOWE: 999</t>
   </si>
   <si>
@@ -96,6 +266,108 @@
     <t>Postępowanie w przypadku awarii</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Postępowanie w przypadku pożaru:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t xml:space="preserve"> z pkt 5.1 KCH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Odpowiednie środki gaśnicze</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">:  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t>z pkt 5.1 KCH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>Nieodpowiednie środki gaśnicze:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t>z pkt 5.1 KCH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Postępowanie w przypadku niezamierzonego uwolnienia się do środowiska: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t>z pkt. 6.3 KCH</t>
+    </r>
+  </si>
+  <si>
     <t>STRAŻ POŻARNA: 998</t>
   </si>
   <si>
@@ -103,6 +375,57 @@
   </si>
   <si>
     <t>Postępowanie z mieszaniną i magazynowanie</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Postępowanie z produktem: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t>z pkt. 7.1 KCH</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">Magazynowanie: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Arial"/>
+        <charset val="238"/>
+      </rPr>
+      <t>z pkt 7.3 KCH</t>
+    </r>
   </si>
   <si>
     <t>Opracował:</t>
@@ -124,7 +447,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="38">
+  <fonts count="41">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -199,6 +522,19 @@
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -242,13 +578,6 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <u/>
       <sz val="11"/>
       <color rgb="FF0000FF"/>
@@ -391,6 +720,18 @@
       <name val="Calibri"/>
       <charset val="0"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <charset val="238"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
     </font>
   </fonts>
   <fills count="35">
@@ -599,7 +940,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -811,6 +1152,17 @@
         <color auto="1"/>
       </right>
       <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -915,152 +1267,152 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="176" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="177" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="18" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="4" borderId="20" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="21" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="5" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="6" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="23" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="7" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="0" borderId="26" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="5" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="6" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="7" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="32" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="33" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="34" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="33" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="70">
+  <cellXfs count="82">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1174,19 +1526,55 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1201,25 +1589,25 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1228,13 +1616,13 @@
     <xf numFmtId="58" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2252,12 +2640,12 @@
       <c r="G1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="63"/>
-      <c r="J1" s="63"/>
-      <c r="K1" s="64"/>
-      <c r="L1" s="64"/>
-      <c r="M1" s="65"/>
-      <c r="N1" s="65"/>
+      <c r="I1" s="75"/>
+      <c r="J1" s="75"/>
+      <c r="K1" s="76"/>
+      <c r="L1" s="76"/>
+      <c r="M1" s="77"/>
+      <c r="N1" s="77"/>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:14">
       <c r="A2" s="13"/>
@@ -2270,12 +2658,12 @@
       <c r="G2" s="15">
         <v>44501</v>
       </c>
-      <c r="I2" s="63"/>
-      <c r="J2" s="63"/>
-      <c r="K2" s="64"/>
-      <c r="L2" s="64"/>
-      <c r="M2" s="65"/>
-      <c r="N2" s="66"/>
+      <c r="I2" s="75"/>
+      <c r="J2" s="75"/>
+      <c r="K2" s="76"/>
+      <c r="L2" s="76"/>
+      <c r="M2" s="77"/>
+      <c r="N2" s="78"/>
     </row>
     <row r="3" ht="23.4" customHeight="1" spans="1:14">
       <c r="A3" s="16"/>
@@ -2287,12 +2675,12 @@
         <v>4</v>
       </c>
       <c r="G3" s="15"/>
-      <c r="I3" s="63"/>
-      <c r="J3" s="63"/>
-      <c r="K3" s="64"/>
-      <c r="L3" s="64"/>
-      <c r="M3" s="65"/>
-      <c r="N3" s="66"/>
+      <c r="I3" s="75"/>
+      <c r="J3" s="75"/>
+      <c r="K3" s="76"/>
+      <c r="L3" s="76"/>
+      <c r="M3" s="77"/>
+      <c r="N3" s="78"/>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="19"/>
@@ -2302,12 +2690,12 @@
       <c r="E4" s="20"/>
       <c r="F4" s="20"/>
       <c r="G4" s="21"/>
-      <c r="I4" s="67"/>
-      <c r="J4" s="67"/>
-      <c r="K4" s="67"/>
-      <c r="L4" s="67"/>
-      <c r="M4" s="67"/>
-      <c r="N4" s="67"/>
+      <c r="I4" s="79"/>
+      <c r="J4" s="79"/>
+      <c r="K4" s="79"/>
+      <c r="L4" s="79"/>
+      <c r="M4" s="79"/>
+      <c r="N4" s="79"/>
     </row>
     <row r="5" ht="16.05" customHeight="1" spans="1:7">
       <c r="A5" s="22" t="s">
@@ -2550,41 +2938,81 @@
       <c r="G39" s="21"/>
     </row>
     <row r="40" ht="78.6" customHeight="1" spans="1:7">
-      <c r="A40" s="49"/>
-      <c r="G40" s="14"/>
+      <c r="A40" s="49" t="s">
+        <v>17</v>
+      </c>
+      <c r="B40" s="50"/>
+      <c r="C40" s="50"/>
+      <c r="D40" s="50"/>
+      <c r="E40" s="50"/>
+      <c r="F40" s="50"/>
+      <c r="G40" s="51"/>
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:7">
-      <c r="A41" s="49"/>
-      <c r="G41" s="14"/>
+      <c r="A41" s="49" t="s">
+        <v>18</v>
+      </c>
+      <c r="B41" s="50"/>
+      <c r="C41" s="50"/>
+      <c r="D41" s="50"/>
+      <c r="E41" s="50"/>
+      <c r="F41" s="50"/>
+      <c r="G41" s="51"/>
     </row>
     <row r="42" ht="14.4" customHeight="1" spans="1:7">
-      <c r="A42" s="49"/>
-      <c r="G42" s="14"/>
+      <c r="A42" s="49" t="s">
+        <v>19</v>
+      </c>
+      <c r="B42" s="50"/>
+      <c r="C42" s="50"/>
+      <c r="D42" s="50"/>
+      <c r="E42" s="50"/>
+      <c r="F42" s="50"/>
+      <c r="G42" s="51"/>
     </row>
     <row r="43" ht="28.2" customHeight="1" spans="1:7">
-      <c r="A43" s="49"/>
-      <c r="G43" s="14"/>
+      <c r="A43" s="49" t="s">
+        <v>20</v>
+      </c>
+      <c r="B43" s="50"/>
+      <c r="C43" s="50"/>
+      <c r="D43" s="50"/>
+      <c r="E43" s="50"/>
+      <c r="F43" s="50"/>
+      <c r="G43" s="51"/>
     </row>
     <row r="44" ht="16.2" customHeight="1" spans="1:7">
-      <c r="A44" s="49"/>
-      <c r="G44" s="14"/>
+      <c r="A44" s="49" t="s">
+        <v>21</v>
+      </c>
+      <c r="B44" s="50"/>
+      <c r="C44" s="50"/>
+      <c r="D44" s="50"/>
+      <c r="E44" s="50"/>
+      <c r="F44" s="50"/>
+      <c r="G44" s="51"/>
     </row>
     <row r="45" ht="6" customHeight="1" spans="1:7">
-      <c r="A45" s="40"/>
-      <c r="G45" s="14"/>
+      <c r="A45" s="52"/>
+      <c r="B45" s="53"/>
+      <c r="C45" s="53"/>
+      <c r="D45" s="53"/>
+      <c r="E45" s="53"/>
+      <c r="F45" s="53"/>
+      <c r="G45" s="54"/>
     </row>
     <row r="46" ht="25.8" customHeight="1" spans="1:7">
-      <c r="A46" s="50" t="s">
-        <v>17</v>
-      </c>
-      <c r="D46" s="51" t="s">
-        <v>18</v>
+      <c r="A46" s="55" t="s">
+        <v>22</v>
+      </c>
+      <c r="D46" s="56" t="s">
+        <v>23</v>
       </c>
       <c r="G46" s="14"/>
     </row>
     <row r="47" ht="16.05" customHeight="1" spans="1:7">
       <c r="A47" s="28" t="s">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -2594,33 +3022,61 @@
       <c r="G47" s="21"/>
     </row>
     <row r="48" ht="14.4" customHeight="1" spans="1:7">
-      <c r="A48" s="37"/>
-      <c r="G48" s="14"/>
+      <c r="A48" s="57" t="s">
+        <v>25</v>
+      </c>
+      <c r="B48" s="58"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="58"/>
+      <c r="E48" s="58"/>
+      <c r="F48" s="58"/>
+      <c r="G48" s="59"/>
     </row>
     <row r="49" ht="25.8" customHeight="1" spans="1:7">
-      <c r="A49" s="37"/>
-      <c r="G49" s="14"/>
+      <c r="A49" s="57" t="s">
+        <v>26</v>
+      </c>
+      <c r="B49" s="58"/>
+      <c r="C49" s="58"/>
+      <c r="D49" s="58"/>
+      <c r="E49" s="58"/>
+      <c r="F49" s="58"/>
+      <c r="G49" s="59"/>
     </row>
     <row r="50" ht="16.8" customHeight="1" spans="1:7">
-      <c r="A50" s="37"/>
-      <c r="G50" s="14"/>
+      <c r="A50" s="57" t="s">
+        <v>27</v>
+      </c>
+      <c r="B50" s="58"/>
+      <c r="C50" s="58"/>
+      <c r="D50" s="58"/>
+      <c r="E50" s="58"/>
+      <c r="F50" s="58"/>
+      <c r="G50" s="59"/>
     </row>
     <row r="51" ht="67.8" customHeight="1" spans="1:7">
-      <c r="A51" s="52"/>
-      <c r="G51" s="14"/>
+      <c r="A51" s="60" t="s">
+        <v>28</v>
+      </c>
+      <c r="B51" s="61"/>
+      <c r="C51" s="61"/>
+      <c r="D51" s="61"/>
+      <c r="E51" s="61"/>
+      <c r="F51" s="61"/>
+      <c r="G51" s="62"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:7">
-      <c r="A52" s="50" t="s">
-        <v>20</v>
-      </c>
-      <c r="E52" s="51" t="s">
-        <v>21</v>
+      <c r="A52" s="55" t="s">
+        <v>29</v>
+      </c>
+      <c r="E52" s="56" t="s">
+        <v>30</v>
       </c>
       <c r="G52" s="14"/>
     </row>
     <row r="53" ht="16.05" customHeight="1" spans="1:7">
       <c r="A53" s="28" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B53" s="20"/>
       <c r="C53" s="20"/>
@@ -2630,120 +3086,129 @@
       <c r="G53" s="21"/>
     </row>
     <row r="54" ht="79.8" customHeight="1" spans="1:7">
-      <c r="A54" s="53"/>
-      <c r="B54" s="11"/>
-      <c r="C54" s="11"/>
-      <c r="D54" s="11"/>
-      <c r="E54" s="11"/>
-      <c r="F54" s="11"/>
-      <c r="G54" s="9"/>
+      <c r="A54" s="63" t="s">
+        <v>32</v>
+      </c>
+      <c r="B54" s="64"/>
+      <c r="C54" s="64"/>
+      <c r="D54" s="64"/>
+      <c r="E54" s="64"/>
+      <c r="F54" s="64"/>
+      <c r="G54" s="65"/>
     </row>
     <row r="55" ht="49.2" customHeight="1" spans="1:7">
-      <c r="A55" s="49"/>
-      <c r="G55" s="14"/>
+      <c r="A55" s="49" t="s">
+        <v>33</v>
+      </c>
+      <c r="B55" s="50"/>
+      <c r="C55" s="50"/>
+      <c r="D55" s="50"/>
+      <c r="E55" s="50"/>
+      <c r="F55" s="50"/>
+      <c r="G55" s="51"/>
     </row>
     <row r="56" ht="9" customHeight="1" spans="1:7">
-      <c r="A56" s="54"/>
-      <c r="B56" s="55"/>
-      <c r="C56" s="55"/>
-      <c r="D56" s="55"/>
-      <c r="E56" s="55"/>
-      <c r="F56" s="55"/>
-      <c r="G56" s="56"/>
+      <c r="A56" s="66"/>
+      <c r="B56" s="67"/>
+      <c r="C56" s="67"/>
+      <c r="D56" s="67"/>
+      <c r="E56" s="67"/>
+      <c r="F56" s="67"/>
+      <c r="G56" s="68"/>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="57" t="s">
-        <v>23</v>
+      <c r="A57" s="69" t="s">
+        <v>34</v>
       </c>
       <c r="B57" s="21"/>
-      <c r="C57" s="57" t="s">
-        <v>24</v>
+      <c r="C57" s="69" t="s">
+        <v>35</v>
       </c>
       <c r="D57" s="20"/>
       <c r="E57" s="21"/>
-      <c r="F57" s="57" t="s">
-        <v>25</v>
+      <c r="F57" s="69" t="s">
+        <v>36</v>
       </c>
       <c r="G57" s="21"/>
     </row>
     <row r="58" ht="40.95" customHeight="1" spans="1:7">
-      <c r="A58" s="58"/>
+      <c r="A58" s="70"/>
       <c r="B58" s="21"/>
-      <c r="C58" s="59"/>
+      <c r="C58" s="71"/>
       <c r="D58" s="20"/>
       <c r="E58" s="21"/>
-      <c r="F58" s="59"/>
+      <c r="F58" s="71"/>
       <c r="G58" s="21"/>
     </row>
     <row r="59" hidden="1" spans="1:11">
-      <c r="A59" s="60"/>
-      <c r="B59" s="60"/>
-      <c r="C59" s="60"/>
-      <c r="D59" s="60"/>
-      <c r="E59" s="60"/>
-      <c r="F59" s="60"/>
-      <c r="G59" s="60"/>
-      <c r="K59" s="68"/>
+      <c r="A59" s="72"/>
+      <c r="B59" s="72"/>
+      <c r="C59" s="72"/>
+      <c r="D59" s="72"/>
+      <c r="E59" s="72"/>
+      <c r="F59" s="72"/>
+      <c r="G59" s="72"/>
+      <c r="K59" s="80"/>
     </row>
     <row r="60" hidden="1" spans="1:1">
-      <c r="A60" s="61"/>
+      <c r="A60" s="73"/>
     </row>
     <row r="61" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A61" s="62"/>
+      <c r="A61" s="74"/>
     </row>
     <row r="62" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A62" s="62"/>
+      <c r="A62" s="74"/>
     </row>
     <row r="63" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A63" s="62"/>
+      <c r="A63" s="74"/>
     </row>
     <row r="64" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A64" s="62"/>
+      <c r="A64" s="74"/>
     </row>
     <row r="65" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A65" s="62"/>
+      <c r="A65" s="74"/>
     </row>
     <row r="66" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A66" s="62"/>
+      <c r="A66" s="74"/>
     </row>
     <row r="67" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A67" s="62"/>
+      <c r="A67" s="74"/>
     </row>
     <row r="68" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A68" s="62"/>
+      <c r="A68" s="74"/>
     </row>
     <row r="69" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A69" s="62"/>
+      <c r="A69" s="74"/>
     </row>
     <row r="70" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A70" s="62"/>
+      <c r="A70" s="74"/>
     </row>
     <row r="71" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A71" s="62"/>
+      <c r="A71" s="74"/>
     </row>
     <row r="72" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A72" s="62"/>
+      <c r="A72" s="74"/>
     </row>
     <row r="73" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A73" s="62"/>
+      <c r="A73" s="74"/>
     </row>
     <row r="74" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A74" s="62"/>
+      <c r="A74" s="74"/>
     </row>
     <row r="75" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A75" s="62"/>
+      <c r="A75" s="74"/>
     </row>
     <row r="76" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A76" s="62"/>
+      <c r="A76" s="74"/>
     </row>
     <row r="77" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A77" s="62"/>
+      <c r="A77" s="74"/>
     </row>
     <row r="78" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A78" s="62"/>
+      <c r="A78" s="74"/>
     </row>
     <row r="79" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A79" s="69"/>
+      <c r="A79" s="81"/>
     </row>
   </sheetData>
   <mergeCells count="67">

</xml_diff>

<commit_message>
Update template with latest headers and layout adjustments
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/wzor.xlsx
+++ b/wzor.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
   <si>
     <t>INSTRUKCJA BHP
 PRZY STOSOWANIU MIESZANIN 
@@ -78,10 +78,94 @@
     <t>Czynności przed rozpoczęciem pracy</t>
   </si>
   <si>
+    <t>Do pracy może być dopuszczony pracownik:</t>
+  </si>
+  <si>
+    <t>-    po przeszkoleniu w zakresie bhp na stanowisku pracy, w wyniku którego stwierdzone zostało przez bezpośredniego przełożonego poznanie bezpiecznych metod pracy,</t>
+  </si>
+  <si>
+    <t>-    po zapoznaniu się z procesem produkcyjnym, wysłuchaniu poleceń i instruktażu bezpośredniego przełożonego, dotyczącego bezpiecznego i prawidłowego wykonywania otrzymanego zadania,</t>
+  </si>
+  <si>
+    <t>-    po zaznajomieniu z kartą charakterystyki stosowanej substancji/mieszaniny niebezpiecznej i instrukcją bezpiecznego stosowania.</t>
+  </si>
+  <si>
+    <t>Czynności przed przystąpieniem do pracy:</t>
+  </si>
+  <si>
+    <t>-    przygotowanie stanowiska pracy,</t>
+  </si>
+  <si>
+    <t>-    przygotowanie i sprawdzenie sprzętu ochronnego,</t>
+  </si>
+  <si>
+    <t>-    włączenie wentylacji ogólnej.</t>
+  </si>
+  <si>
     <t>Czynności w czasie pracy</t>
   </si>
   <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">-    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">stosować odpowiednie środki ochrony indywidualnej, </t>
+    </r>
+  </si>
+  <si>
+    <t>-    zabezpieczyć produkt przed rozlaniem się, stosować tylko bezpieczne metody pracy i wykonywać wyłącznie zadania polecone przez swojego bezpośredniego przełożonego, unikać zanieczyszczenia oczu i skóry,</t>
+  </si>
+  <si>
+    <t>-    każdorazowo po zakończeniu pracy z substancją/mieszaniną niebezpieczną umyć dokładnie ręce, stosować krem ochronny,</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t xml:space="preserve">-    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <charset val="134"/>
+      </rPr>
+      <t>podczas pracy nie pić, nie jeść, nie zażywać leków, nie palić,</t>
+    </r>
+  </si>
+  <si>
+    <t>-    unikać wdychania oparów,</t>
+  </si>
+  <si>
+    <t>-    dbać o ład i porządek na stanowisku pracy, przestrzegać zasad higieny osobistej.</t>
+  </si>
+  <si>
     <t>Czynności po zakończeniu pracy</t>
+  </si>
+  <si>
+    <t>- uprzątnąć i uporządkować miejsca pracy, sprawdzić czy pojemnik zawierający substancję/mieszaninę niebezpieczną jest szczelnie zamknięty i odłożony na swoje miejsce, upewnić się czy pozostawione miejsce pracy nie stworzy żadnych zagrożeń dla otoczenia, sprawdzić środki ochrony indywidualnej i odłożyć je na wyznaczone miejsce,</t>
+  </si>
+  <si>
+    <t>- w przypadku zanieczyszczenia środkiem ubranie przekazać do prania, po zakończeniu pracy z substancją/mieszaniną niebezpieczną dokładnie umyć ręce i twarz, przekazać swojemu bezpośredniemu przełożonemu informację o zakończeniu pracy.</t>
   </si>
   <si>
     <t>Pierwsza pomoc</t>
@@ -447,7 +531,7 @@
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
   </numFmts>
-  <fonts count="41">
+  <fonts count="43">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -514,13 +598,8 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <charset val="134"/>
-    </font>
-    <font>
-      <sz val="10"/>
+      <b/>
+      <sz val="12"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="134"/>
@@ -533,8 +612,20 @@
       <charset val="134"/>
     </font>
     <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -723,13 +814,20 @@
     </font>
     <font>
       <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="10"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
       <charset val="238"/>
     </font>
     <font>
+      <b/>
       <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <charset val="134"/>
     </font>
@@ -940,7 +1038,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="29">
+  <borders count="30">
     <border>
       <left/>
       <right/>
@@ -1153,6 +1251,19 @@
       </right>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -1282,137 +1393,137 @@
     <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="21" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="22" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="22" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="25" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="23" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="5" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="29" fillId="6" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="6" borderId="24" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="31" fillId="7" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="32" fillId="0" borderId="27" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="24" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="5" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="6" borderId="26" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="31" fillId="6" borderId="25" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="7" borderId="27" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="33" fillId="0" borderId="28" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="34" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="36" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="37" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="29" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="36" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="39" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="38" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="82">
+  <cellXfs count="96">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -1490,31 +1601,73 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1526,55 +1679,55 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1589,41 +1742,44 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="58" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="58" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" quotePrefix="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1694,6 +1850,99 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>523044</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>182316</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>116644</xdr:colOff>
+      <xdr:row>33</xdr:row>
+      <xdr:rowOff>250261</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Obraz 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId1" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="522605" y="7872730"/>
+          <a:ext cx="689610" cy="723265"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>519545</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>76200</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>1</xdr:col>
+      <xdr:colOff>112510</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>136525</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Obraz 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="519430" y="7103745"/>
+          <a:ext cx="688975" cy="723265"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
@@ -2640,12 +2889,12 @@
       <c r="G1" s="12" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="75"/>
-      <c r="J1" s="75"/>
-      <c r="K1" s="76"/>
-      <c r="L1" s="76"/>
-      <c r="M1" s="77"/>
-      <c r="N1" s="77"/>
+      <c r="I1" s="89"/>
+      <c r="J1" s="89"/>
+      <c r="K1" s="90"/>
+      <c r="L1" s="90"/>
+      <c r="M1" s="91"/>
+      <c r="N1" s="91"/>
     </row>
     <row r="2" ht="15" customHeight="1" spans="1:14">
       <c r="A2" s="13"/>
@@ -2658,12 +2907,12 @@
       <c r="G2" s="15">
         <v>44501</v>
       </c>
-      <c r="I2" s="75"/>
-      <c r="J2" s="75"/>
-      <c r="K2" s="76"/>
-      <c r="L2" s="76"/>
-      <c r="M2" s="77"/>
-      <c r="N2" s="78"/>
+      <c r="I2" s="89"/>
+      <c r="J2" s="89"/>
+      <c r="K2" s="90"/>
+      <c r="L2" s="90"/>
+      <c r="M2" s="91"/>
+      <c r="N2" s="92"/>
     </row>
     <row r="3" ht="23.4" customHeight="1" spans="1:14">
       <c r="A3" s="16"/>
@@ -2675,12 +2924,12 @@
         <v>4</v>
       </c>
       <c r="G3" s="15"/>
-      <c r="I3" s="75"/>
-      <c r="J3" s="75"/>
-      <c r="K3" s="76"/>
-      <c r="L3" s="76"/>
-      <c r="M3" s="77"/>
-      <c r="N3" s="78"/>
+      <c r="I3" s="89"/>
+      <c r="J3" s="89"/>
+      <c r="K3" s="90"/>
+      <c r="L3" s="90"/>
+      <c r="M3" s="91"/>
+      <c r="N3" s="92"/>
     </row>
     <row r="4" spans="1:14">
       <c r="A4" s="19"/>
@@ -2690,12 +2939,12 @@
       <c r="E4" s="20"/>
       <c r="F4" s="20"/>
       <c r="G4" s="21"/>
-      <c r="I4" s="79"/>
-      <c r="J4" s="79"/>
-      <c r="K4" s="79"/>
-      <c r="L4" s="79"/>
-      <c r="M4" s="79"/>
-      <c r="N4" s="79"/>
+      <c r="I4" s="93"/>
+      <c r="J4" s="93"/>
+      <c r="K4" s="93"/>
+      <c r="L4" s="93"/>
+      <c r="M4" s="93"/>
+      <c r="N4" s="93"/>
     </row>
     <row r="5" ht="16.05" customHeight="1" spans="1:7">
       <c r="A5" s="22" t="s">
@@ -2807,128 +3056,235 @@
       <c r="G17" s="17"/>
     </row>
     <row r="18" ht="16.05" customHeight="1" spans="1:7">
-      <c r="A18" s="28" t="s">
+      <c r="A18" s="37" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="21"/>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="39"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="37"/>
-      <c r="G19" s="14"/>
+      <c r="A19" s="40" t="s">
+        <v>14</v>
+      </c>
+      <c r="B19" s="41"/>
+      <c r="C19" s="41"/>
+      <c r="D19" s="41"/>
+      <c r="E19" s="41"/>
+      <c r="F19" s="41"/>
+      <c r="G19" s="42"/>
     </row>
     <row r="20" ht="25.2" customHeight="1" spans="1:7">
-      <c r="A20" s="38"/>
-      <c r="G20" s="14"/>
+      <c r="A20" s="43" t="s">
+        <v>15</v>
+      </c>
+      <c r="B20" s="44"/>
+      <c r="C20" s="44"/>
+      <c r="D20" s="44"/>
+      <c r="E20" s="44"/>
+      <c r="F20" s="44"/>
+      <c r="G20" s="45"/>
     </row>
     <row r="21" ht="25.2" customHeight="1" spans="1:7">
-      <c r="A21" s="38"/>
-      <c r="G21" s="14"/>
+      <c r="A21" s="43" t="s">
+        <v>16</v>
+      </c>
+      <c r="B21" s="44"/>
+      <c r="C21" s="44"/>
+      <c r="D21" s="44"/>
+      <c r="E21" s="44"/>
+      <c r="F21" s="44"/>
+      <c r="G21" s="45"/>
     </row>
     <row r="22" ht="28.8" customHeight="1" spans="1:7">
-      <c r="A22" s="38"/>
-      <c r="G22" s="14"/>
+      <c r="A22" s="43" t="s">
+        <v>17</v>
+      </c>
+      <c r="B22" s="44"/>
+      <c r="C22" s="44"/>
+      <c r="D22" s="44"/>
+      <c r="E22" s="44"/>
+      <c r="F22" s="44"/>
+      <c r="G22" s="45"/>
     </row>
     <row r="23" ht="13.8" customHeight="1" spans="1:7">
-      <c r="A23" s="37"/>
-      <c r="G23" s="14"/>
+      <c r="A23" s="40" t="s">
+        <v>18</v>
+      </c>
+      <c r="B23" s="41"/>
+      <c r="C23" s="41"/>
+      <c r="D23" s="41"/>
+      <c r="E23" s="41"/>
+      <c r="F23" s="41"/>
+      <c r="G23" s="42"/>
     </row>
     <row r="24" ht="13.8" customHeight="1" spans="1:7">
-      <c r="A24" s="39"/>
-      <c r="G24" s="14"/>
+      <c r="A24" s="46" t="s">
+        <v>19</v>
+      </c>
+      <c r="B24" s="47"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="48"/>
     </row>
     <row r="25" ht="13.8" customHeight="1" spans="1:7">
-      <c r="A25" s="39"/>
-      <c r="G25" s="14"/>
+      <c r="A25" s="46" t="s">
+        <v>20</v>
+      </c>
+      <c r="B25" s="47"/>
+      <c r="C25" s="47"/>
+      <c r="D25" s="47"/>
+      <c r="E25" s="47"/>
+      <c r="F25" s="47"/>
+      <c r="G25" s="48"/>
     </row>
     <row r="26" ht="13.8" customHeight="1" spans="1:7">
-      <c r="A26" s="39"/>
-      <c r="G26" s="14"/>
+      <c r="A26" s="46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B26" s="47"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="48"/>
     </row>
     <row r="27" ht="6" customHeight="1" spans="1:7">
-      <c r="A27" s="40"/>
-      <c r="G27" s="14"/>
+      <c r="A27" s="49"/>
+      <c r="B27" s="50"/>
+      <c r="C27" s="50"/>
+      <c r="D27" s="50"/>
+      <c r="E27" s="50"/>
+      <c r="F27" s="50"/>
+      <c r="G27" s="51"/>
     </row>
     <row r="28" ht="16.05" customHeight="1" spans="1:7">
-      <c r="A28" s="28" t="s">
-        <v>14</v>
-      </c>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="21"/>
+      <c r="A28" s="37" t="s">
+        <v>22</v>
+      </c>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="39"/>
     </row>
     <row r="29" ht="13.2" customHeight="1" spans="1:7">
-      <c r="A29" s="41"/>
-      <c r="C29" s="42"/>
-      <c r="G29" s="14"/>
+      <c r="A29" s="52"/>
+      <c r="B29" s="53"/>
+      <c r="C29" s="47" t="s">
+        <v>23</v>
+      </c>
+      <c r="D29" s="47"/>
+      <c r="E29" s="47"/>
+      <c r="F29" s="47"/>
+      <c r="G29" s="48"/>
     </row>
     <row r="30" ht="39" customHeight="1" spans="1:7">
-      <c r="A30" s="13"/>
-      <c r="C30" s="43"/>
-      <c r="G30" s="14"/>
+      <c r="A30" s="52"/>
+      <c r="B30" s="53"/>
+      <c r="C30" s="44" t="s">
+        <v>24</v>
+      </c>
+      <c r="D30" s="44"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="44"/>
+      <c r="G30" s="45"/>
     </row>
     <row r="31" ht="25.2" customHeight="1" spans="1:7">
-      <c r="A31" s="13"/>
-      <c r="C31" s="43"/>
-      <c r="G31" s="14"/>
+      <c r="A31" s="52"/>
+      <c r="B31" s="53"/>
+      <c r="C31" s="44" t="s">
+        <v>25</v>
+      </c>
+      <c r="D31" s="44"/>
+      <c r="E31" s="44"/>
+      <c r="F31" s="44"/>
+      <c r="G31" s="45"/>
     </row>
     <row r="32" ht="13.8" customHeight="1" spans="1:7">
-      <c r="A32" s="13"/>
-      <c r="C32" s="44"/>
-      <c r="G32" s="14"/>
+      <c r="A32" s="52"/>
+      <c r="B32" s="53"/>
+      <c r="C32" s="54" t="s">
+        <v>26</v>
+      </c>
+      <c r="D32" s="54"/>
+      <c r="E32" s="54"/>
+      <c r="F32" s="54"/>
+      <c r="G32" s="55"/>
     </row>
     <row r="33" ht="12.6" customHeight="1" spans="1:7">
-      <c r="A33" s="13"/>
-      <c r="C33" s="44"/>
-      <c r="G33" s="14"/>
+      <c r="A33" s="52"/>
+      <c r="B33" s="53"/>
+      <c r="C33" s="54" t="s">
+        <v>27</v>
+      </c>
+      <c r="D33" s="54"/>
+      <c r="E33" s="54"/>
+      <c r="F33" s="54"/>
+      <c r="G33" s="55"/>
     </row>
     <row r="34" ht="27.9" customHeight="1" spans="1:7">
-      <c r="A34" s="16"/>
-      <c r="B34" s="18"/>
-      <c r="C34" s="45"/>
-      <c r="D34" s="18"/>
-      <c r="E34" s="18"/>
-      <c r="F34" s="18"/>
-      <c r="G34" s="17"/>
+      <c r="A34" s="56"/>
+      <c r="B34" s="57"/>
+      <c r="C34" s="58" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="58"/>
+      <c r="E34" s="58"/>
+      <c r="F34" s="58"/>
+      <c r="G34" s="59"/>
     </row>
     <row r="35" ht="16.05" customHeight="1" spans="1:7">
-      <c r="A35" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="B35" s="20"/>
-      <c r="C35" s="20"/>
-      <c r="D35" s="20"/>
-      <c r="E35" s="20"/>
-      <c r="F35" s="20"/>
-      <c r="G35" s="21"/>
+      <c r="A35" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="B35" s="38"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="39"/>
     </row>
     <row r="36" ht="41.4" customHeight="1" spans="1:7">
-      <c r="A36" s="38"/>
-      <c r="G36" s="14"/>
+      <c r="A36" s="96" t="s">
+        <v>30</v>
+      </c>
+      <c r="B36" s="44"/>
+      <c r="C36" s="44"/>
+      <c r="D36" s="44"/>
+      <c r="E36" s="44"/>
+      <c r="F36" s="44"/>
+      <c r="G36" s="45"/>
     </row>
     <row r="37" ht="38.4" customHeight="1" spans="1:7">
-      <c r="A37" s="38"/>
-      <c r="G37" s="14"/>
+      <c r="A37" s="96" t="s">
+        <v>31</v>
+      </c>
+      <c r="B37" s="44"/>
+      <c r="C37" s="44"/>
+      <c r="D37" s="44"/>
+      <c r="E37" s="44"/>
+      <c r="F37" s="44"/>
+      <c r="G37" s="45"/>
     </row>
     <row r="38" ht="6" customHeight="1" spans="1:7">
-      <c r="A38" s="46"/>
-      <c r="B38" s="47"/>
-      <c r="C38" s="47"/>
-      <c r="D38" s="47"/>
-      <c r="E38" s="47"/>
-      <c r="F38" s="47"/>
-      <c r="G38" s="48"/>
+      <c r="A38" s="60"/>
+      <c r="B38" s="61"/>
+      <c r="C38" s="61"/>
+      <c r="D38" s="61"/>
+      <c r="E38" s="61"/>
+      <c r="F38" s="61"/>
+      <c r="G38" s="62"/>
     </row>
     <row r="39" ht="15.6" customHeight="1" spans="1:7">
       <c r="A39" s="28" t="s">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="B39" s="20"/>
       <c r="C39" s="20"/>
@@ -2938,81 +3294,81 @@
       <c r="G39" s="21"/>
     </row>
     <row r="40" ht="78.6" customHeight="1" spans="1:7">
-      <c r="A40" s="49" t="s">
-        <v>17</v>
-      </c>
-      <c r="B40" s="50"/>
-      <c r="C40" s="50"/>
-      <c r="D40" s="50"/>
-      <c r="E40" s="50"/>
-      <c r="F40" s="50"/>
-      <c r="G40" s="51"/>
+      <c r="A40" s="63" t="s">
+        <v>33</v>
+      </c>
+      <c r="B40" s="64"/>
+      <c r="C40" s="64"/>
+      <c r="D40" s="64"/>
+      <c r="E40" s="64"/>
+      <c r="F40" s="64"/>
+      <c r="G40" s="65"/>
     </row>
     <row r="41" ht="24" customHeight="1" spans="1:7">
-      <c r="A41" s="49" t="s">
-        <v>18</v>
-      </c>
-      <c r="B41" s="50"/>
-      <c r="C41" s="50"/>
-      <c r="D41" s="50"/>
-      <c r="E41" s="50"/>
-      <c r="F41" s="50"/>
-      <c r="G41" s="51"/>
+      <c r="A41" s="63" t="s">
+        <v>34</v>
+      </c>
+      <c r="B41" s="64"/>
+      <c r="C41" s="64"/>
+      <c r="D41" s="64"/>
+      <c r="E41" s="64"/>
+      <c r="F41" s="64"/>
+      <c r="G41" s="65"/>
     </row>
     <row r="42" ht="14.4" customHeight="1" spans="1:7">
-      <c r="A42" s="49" t="s">
-        <v>19</v>
-      </c>
-      <c r="B42" s="50"/>
-      <c r="C42" s="50"/>
-      <c r="D42" s="50"/>
-      <c r="E42" s="50"/>
-      <c r="F42" s="50"/>
-      <c r="G42" s="51"/>
+      <c r="A42" s="63" t="s">
+        <v>35</v>
+      </c>
+      <c r="B42" s="64"/>
+      <c r="C42" s="64"/>
+      <c r="D42" s="64"/>
+      <c r="E42" s="64"/>
+      <c r="F42" s="64"/>
+      <c r="G42" s="65"/>
     </row>
     <row r="43" ht="28.2" customHeight="1" spans="1:7">
-      <c r="A43" s="49" t="s">
-        <v>20</v>
-      </c>
-      <c r="B43" s="50"/>
-      <c r="C43" s="50"/>
-      <c r="D43" s="50"/>
-      <c r="E43" s="50"/>
-      <c r="F43" s="50"/>
-      <c r="G43" s="51"/>
+      <c r="A43" s="63" t="s">
+        <v>36</v>
+      </c>
+      <c r="B43" s="64"/>
+      <c r="C43" s="64"/>
+      <c r="D43" s="64"/>
+      <c r="E43" s="64"/>
+      <c r="F43" s="64"/>
+      <c r="G43" s="65"/>
     </row>
     <row r="44" ht="16.2" customHeight="1" spans="1:7">
-      <c r="A44" s="49" t="s">
-        <v>21</v>
-      </c>
-      <c r="B44" s="50"/>
-      <c r="C44" s="50"/>
-      <c r="D44" s="50"/>
-      <c r="E44" s="50"/>
-      <c r="F44" s="50"/>
-      <c r="G44" s="51"/>
+      <c r="A44" s="63" t="s">
+        <v>37</v>
+      </c>
+      <c r="B44" s="64"/>
+      <c r="C44" s="64"/>
+      <c r="D44" s="64"/>
+      <c r="E44" s="64"/>
+      <c r="F44" s="64"/>
+      <c r="G44" s="65"/>
     </row>
     <row r="45" ht="6" customHeight="1" spans="1:7">
-      <c r="A45" s="52"/>
-      <c r="B45" s="53"/>
-      <c r="C45" s="53"/>
-      <c r="D45" s="53"/>
-      <c r="E45" s="53"/>
-      <c r="F45" s="53"/>
-      <c r="G45" s="54"/>
+      <c r="A45" s="66"/>
+      <c r="B45" s="67"/>
+      <c r="C45" s="67"/>
+      <c r="D45" s="67"/>
+      <c r="E45" s="67"/>
+      <c r="F45" s="67"/>
+      <c r="G45" s="68"/>
     </row>
     <row r="46" ht="25.8" customHeight="1" spans="1:7">
-      <c r="A46" s="55" t="s">
-        <v>22</v>
-      </c>
-      <c r="D46" s="56" t="s">
-        <v>23</v>
+      <c r="A46" s="69" t="s">
+        <v>38</v>
+      </c>
+      <c r="D46" s="70" t="s">
+        <v>39</v>
       </c>
       <c r="G46" s="14"/>
     </row>
     <row r="47" ht="16.05" customHeight="1" spans="1:7">
       <c r="A47" s="28" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="B47" s="20"/>
       <c r="C47" s="20"/>
@@ -3022,61 +3378,61 @@
       <c r="G47" s="21"/>
     </row>
     <row r="48" ht="14.4" customHeight="1" spans="1:7">
-      <c r="A48" s="57" t="s">
-        <v>25</v>
-      </c>
-      <c r="B48" s="58"/>
-      <c r="C48" s="58"/>
-      <c r="D48" s="58"/>
-      <c r="E48" s="58"/>
-      <c r="F48" s="58"/>
-      <c r="G48" s="59"/>
+      <c r="A48" s="71" t="s">
+        <v>41</v>
+      </c>
+      <c r="B48" s="72"/>
+      <c r="C48" s="72"/>
+      <c r="D48" s="72"/>
+      <c r="E48" s="72"/>
+      <c r="F48" s="72"/>
+      <c r="G48" s="73"/>
     </row>
     <row r="49" ht="25.8" customHeight="1" spans="1:7">
-      <c r="A49" s="57" t="s">
-        <v>26</v>
-      </c>
-      <c r="B49" s="58"/>
-      <c r="C49" s="58"/>
-      <c r="D49" s="58"/>
-      <c r="E49" s="58"/>
-      <c r="F49" s="58"/>
-      <c r="G49" s="59"/>
+      <c r="A49" s="71" t="s">
+        <v>42</v>
+      </c>
+      <c r="B49" s="72"/>
+      <c r="C49" s="72"/>
+      <c r="D49" s="72"/>
+      <c r="E49" s="72"/>
+      <c r="F49" s="72"/>
+      <c r="G49" s="73"/>
     </row>
     <row r="50" ht="16.8" customHeight="1" spans="1:7">
-      <c r="A50" s="57" t="s">
-        <v>27</v>
-      </c>
-      <c r="B50" s="58"/>
-      <c r="C50" s="58"/>
-      <c r="D50" s="58"/>
-      <c r="E50" s="58"/>
-      <c r="F50" s="58"/>
-      <c r="G50" s="59"/>
+      <c r="A50" s="71" t="s">
+        <v>43</v>
+      </c>
+      <c r="B50" s="72"/>
+      <c r="C50" s="72"/>
+      <c r="D50" s="72"/>
+      <c r="E50" s="72"/>
+      <c r="F50" s="72"/>
+      <c r="G50" s="73"/>
     </row>
     <row r="51" ht="67.8" customHeight="1" spans="1:7">
-      <c r="A51" s="60" t="s">
-        <v>28</v>
-      </c>
-      <c r="B51" s="61"/>
-      <c r="C51" s="61"/>
-      <c r="D51" s="61"/>
-      <c r="E51" s="61"/>
-      <c r="F51" s="61"/>
-      <c r="G51" s="62"/>
+      <c r="A51" s="74" t="s">
+        <v>44</v>
+      </c>
+      <c r="B51" s="75"/>
+      <c r="C51" s="75"/>
+      <c r="D51" s="75"/>
+      <c r="E51" s="75"/>
+      <c r="F51" s="75"/>
+      <c r="G51" s="76"/>
     </row>
     <row r="52" ht="18" customHeight="1" spans="1:7">
-      <c r="A52" s="55" t="s">
-        <v>29</v>
-      </c>
-      <c r="E52" s="56" t="s">
-        <v>30</v>
+      <c r="A52" s="69" t="s">
+        <v>45</v>
+      </c>
+      <c r="E52" s="70" t="s">
+        <v>46</v>
       </c>
       <c r="G52" s="14"/>
     </row>
     <row r="53" ht="16.05" customHeight="1" spans="1:7">
       <c r="A53" s="28" t="s">
-        <v>31</v>
+        <v>47</v>
       </c>
       <c r="B53" s="20"/>
       <c r="C53" s="20"/>
@@ -3086,129 +3442,129 @@
       <c r="G53" s="21"/>
     </row>
     <row r="54" ht="79.8" customHeight="1" spans="1:7">
-      <c r="A54" s="63" t="s">
-        <v>32</v>
-      </c>
-      <c r="B54" s="64"/>
-      <c r="C54" s="64"/>
-      <c r="D54" s="64"/>
-      <c r="E54" s="64"/>
-      <c r="F54" s="64"/>
-      <c r="G54" s="65"/>
+      <c r="A54" s="77" t="s">
+        <v>48</v>
+      </c>
+      <c r="B54" s="78"/>
+      <c r="C54" s="78"/>
+      <c r="D54" s="78"/>
+      <c r="E54" s="78"/>
+      <c r="F54" s="78"/>
+      <c r="G54" s="79"/>
     </row>
     <row r="55" ht="49.2" customHeight="1" spans="1:7">
-      <c r="A55" s="49" t="s">
-        <v>33</v>
-      </c>
-      <c r="B55" s="50"/>
-      <c r="C55" s="50"/>
-      <c r="D55" s="50"/>
-      <c r="E55" s="50"/>
-      <c r="F55" s="50"/>
-      <c r="G55" s="51"/>
+      <c r="A55" s="63" t="s">
+        <v>49</v>
+      </c>
+      <c r="B55" s="64"/>
+      <c r="C55" s="64"/>
+      <c r="D55" s="64"/>
+      <c r="E55" s="64"/>
+      <c r="F55" s="64"/>
+      <c r="G55" s="65"/>
     </row>
     <row r="56" ht="9" customHeight="1" spans="1:7">
-      <c r="A56" s="66"/>
-      <c r="B56" s="67"/>
-      <c r="C56" s="67"/>
-      <c r="D56" s="67"/>
-      <c r="E56" s="67"/>
-      <c r="F56" s="67"/>
-      <c r="G56" s="68"/>
+      <c r="A56" s="80"/>
+      <c r="B56" s="81"/>
+      <c r="C56" s="81"/>
+      <c r="D56" s="81"/>
+      <c r="E56" s="81"/>
+      <c r="F56" s="81"/>
+      <c r="G56" s="82"/>
     </row>
     <row r="57" spans="1:7">
-      <c r="A57" s="69" t="s">
-        <v>34</v>
+      <c r="A57" s="83" t="s">
+        <v>50</v>
       </c>
       <c r="B57" s="21"/>
-      <c r="C57" s="69" t="s">
-        <v>35</v>
+      <c r="C57" s="83" t="s">
+        <v>51</v>
       </c>
       <c r="D57" s="20"/>
       <c r="E57" s="21"/>
-      <c r="F57" s="69" t="s">
-        <v>36</v>
+      <c r="F57" s="83" t="s">
+        <v>52</v>
       </c>
       <c r="G57" s="21"/>
     </row>
     <row r="58" ht="40.95" customHeight="1" spans="1:7">
-      <c r="A58" s="70"/>
+      <c r="A58" s="84"/>
       <c r="B58" s="21"/>
-      <c r="C58" s="71"/>
+      <c r="C58" s="85"/>
       <c r="D58" s="20"/>
       <c r="E58" s="21"/>
-      <c r="F58" s="71"/>
+      <c r="F58" s="85"/>
       <c r="G58" s="21"/>
     </row>
     <row r="59" hidden="1" spans="1:11">
-      <c r="A59" s="72"/>
-      <c r="B59" s="72"/>
-      <c r="C59" s="72"/>
-      <c r="D59" s="72"/>
-      <c r="E59" s="72"/>
-      <c r="F59" s="72"/>
-      <c r="G59" s="72"/>
-      <c r="K59" s="80"/>
+      <c r="A59" s="86"/>
+      <c r="B59" s="86"/>
+      <c r="C59" s="86"/>
+      <c r="D59" s="86"/>
+      <c r="E59" s="86"/>
+      <c r="F59" s="86"/>
+      <c r="G59" s="86"/>
+      <c r="K59" s="94"/>
     </row>
     <row r="60" hidden="1" spans="1:1">
-      <c r="A60" s="73"/>
+      <c r="A60" s="87"/>
     </row>
     <row r="61" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A61" s="74"/>
+      <c r="A61" s="88"/>
     </row>
     <row r="62" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A62" s="74"/>
+      <c r="A62" s="88"/>
     </row>
     <row r="63" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A63" s="74"/>
+      <c r="A63" s="88"/>
     </row>
     <row r="64" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A64" s="74"/>
+      <c r="A64" s="88"/>
     </row>
     <row r="65" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A65" s="74"/>
+      <c r="A65" s="88"/>
     </row>
     <row r="66" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A66" s="74"/>
+      <c r="A66" s="88"/>
     </row>
     <row r="67" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A67" s="74"/>
+      <c r="A67" s="88"/>
     </row>
     <row r="68" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A68" s="74"/>
+      <c r="A68" s="88"/>
     </row>
     <row r="69" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A69" s="74"/>
+      <c r="A69" s="88"/>
     </row>
     <row r="70" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A70" s="74"/>
+      <c r="A70" s="88"/>
     </row>
     <row r="71" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A71" s="74"/>
+      <c r="A71" s="88"/>
     </row>
     <row r="72" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A72" s="74"/>
+      <c r="A72" s="88"/>
     </row>
     <row r="73" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A73" s="74"/>
+      <c r="A73" s="88"/>
     </row>
     <row r="74" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A74" s="74"/>
+      <c r="A74" s="88"/>
     </row>
     <row r="75" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A75" s="74"/>
+      <c r="A75" s="88"/>
     </row>
     <row r="76" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A76" s="74"/>
+      <c r="A76" s="88"/>
     </row>
     <row r="77" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A77" s="74"/>
+      <c r="A77" s="88"/>
     </row>
     <row r="78" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A78" s="74"/>
+      <c r="A78" s="88"/>
     </row>
     <row r="79" ht="15" hidden="1" customHeight="1" spans="1:1">
-      <c r="A79" s="81"/>
+      <c r="A79" s="95"/>
     </row>
   </sheetData>
   <mergeCells count="67">
@@ -3289,6 +3645,7 @@
   <rowBreaks count="1" manualBreakCount="1">
     <brk id="34" max="16383" man="1"/>
   </rowBreaks>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>